<commit_message>
chore: finalize analytics 2026-09-07
</commit_message>
<xml_diff>
--- a/data/excel/statistics_matrices.xlsx
+++ b/data/excel/statistics_matrices.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,9 +87,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -26631,7 +26628,9 @@
           <t>15</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="3" t="n">
+        <v/>
+      </c>
       <c r="E2" s="3" t="n">
         <v>392</v>
       </c>
@@ -26659,7 +26658,9 @@
           <t>19</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n"/>
+      <c r="D3" s="3" t="n">
+        <v/>
+      </c>
       <c r="E3" s="3" t="n">
         <v>392</v>
       </c>
@@ -26687,7 +26688,9 @@
           <t>39</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
+      <c r="D4" s="3" t="n">
+        <v/>
+      </c>
       <c r="E4" s="3" t="n">
         <v>392</v>
       </c>
@@ -70355,7 +70358,9 @@
       <c r="D2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="4" t="n"/>
+      <c r="E2" s="3" t="n">
+        <v/>
+      </c>
       <c r="F2" s="3" t="n">
         <v>392</v>
       </c>
@@ -70393,7 +70398,9 @@
       <c r="D3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="4" t="n"/>
+      <c r="E3" s="3" t="n">
+        <v/>
+      </c>
       <c r="F3" s="3" t="n">
         <v>392</v>
       </c>
@@ -70431,7 +70438,9 @@
       <c r="D4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="4" t="n"/>
+      <c r="E4" s="3" t="n">
+        <v/>
+      </c>
       <c r="F4" s="3" t="n">
         <v>392</v>
       </c>
@@ -70469,7 +70478,9 @@
       <c r="D5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="n"/>
+      <c r="E5" s="3" t="n">
+        <v/>
+      </c>
       <c r="F5" s="3" t="n">
         <v>392</v>
       </c>

</xml_diff>